<commit_message>
New trainings and analyses
</commit_message>
<xml_diff>
--- a/htk_files/results/results_3_states/HMM_Results_3_states.xlsx
+++ b/htk_files/results/results_3_states/HMM_Results_3_states.xlsx
@@ -531,7 +531,7 @@
         <v>66.67</v>
       </c>
       <c r="L2" t="n">
-        <v>55.335</v>
+        <v>55.34</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         <v>63.33</v>
       </c>
       <c r="L3" t="n">
-        <v>53.33199999999999</v>
+        <v>53.33</v>
       </c>
     </row>
     <row r="4">
@@ -611,7 +611,7 @@
         <v>50</v>
       </c>
       <c r="L4" t="n">
-        <v>48.334</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="5">
@@ -651,7 +651,7 @@
         <v>46.67</v>
       </c>
       <c r="L5" t="n">
-        <v>51.66699999999999</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="6">
@@ -691,7 +691,7 @@
         <v>43.33</v>
       </c>
       <c r="L6" t="n">
-        <v>39.999</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -731,7 +731,7 @@
         <v>50</v>
       </c>
       <c r="L7" t="n">
-        <v>51.999</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
@@ -771,7 +771,7 @@
         <v>36.67</v>
       </c>
       <c r="L8" t="n">
-        <v>43.334</v>
+        <v>43.33</v>
       </c>
     </row>
     <row r="9">
@@ -811,7 +811,7 @@
         <v>46.67</v>
       </c>
       <c r="L9" t="n">
-        <v>41.66800000000001</v>
+        <v>41.67</v>
       </c>
     </row>
     <row r="10">
@@ -851,7 +851,7 @@
         <v>63.64</v>
       </c>
       <c r="L10" t="n">
-        <v>60.911</v>
+        <v>60.91</v>
       </c>
     </row>
     <row r="11">
@@ -891,7 +891,7 @@
         <v>60.61</v>
       </c>
       <c r="L11" t="n">
-        <v>56.366</v>
+        <v>56.37</v>
       </c>
     </row>
     <row r="12">
@@ -901,37 +901,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47.63700000000001</v>
+        <v>47.64</v>
       </c>
       <c r="C12" t="n">
-        <v>50.123</v>
+        <v>50.12</v>
       </c>
       <c r="D12" t="n">
-        <v>43.241</v>
+        <v>43.24</v>
       </c>
       <c r="E12" t="n">
-        <v>43.667</v>
+        <v>43.67</v>
       </c>
       <c r="F12" t="n">
-        <v>51.183</v>
+        <v>51.18</v>
       </c>
       <c r="G12" t="n">
-        <v>50.365</v>
+        <v>50.36</v>
       </c>
       <c r="H12" t="n">
-        <v>53.697</v>
+        <v>53.7</v>
       </c>
       <c r="I12" t="n">
-        <v>55.30300000000001</v>
+        <v>55.3</v>
       </c>
       <c r="J12" t="n">
-        <v>54.97000000000001</v>
+        <v>54.97</v>
       </c>
       <c r="K12" t="n">
-        <v>52.759</v>
+        <v>52.76</v>
       </c>
       <c r="L12" t="n">
-        <v>50.2945</v>
+        <v>50.29</v>
       </c>
     </row>
   </sheetData>
@@ -1042,7 +1042,7 @@
         <v>70</v>
       </c>
       <c r="L2" t="n">
-        <v>58.666</v>
+        <v>58.67</v>
       </c>
     </row>
     <row r="3">
@@ -1082,7 +1082,7 @@
         <v>36.67</v>
       </c>
       <c r="L3" t="n">
-        <v>43.999</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -1122,7 +1122,7 @@
         <v>40</v>
       </c>
       <c r="L4" t="n">
-        <v>38.99999999999999</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -1162,7 +1162,7 @@
         <v>63.33</v>
       </c>
       <c r="L5" t="n">
-        <v>46.333</v>
+        <v>46.33</v>
       </c>
     </row>
     <row r="6">
@@ -1202,7 +1202,7 @@
         <v>43.33</v>
       </c>
       <c r="L6" t="n">
-        <v>39.666</v>
+        <v>39.67</v>
       </c>
     </row>
     <row r="7">
@@ -1242,7 +1242,7 @@
         <v>60</v>
       </c>
       <c r="L7" t="n">
-        <v>50.334</v>
+        <v>50.33</v>
       </c>
     </row>
     <row r="8">
@@ -1282,7 +1282,7 @@
         <v>30</v>
       </c>
       <c r="L8" t="n">
-        <v>38.333</v>
+        <v>38.33</v>
       </c>
     </row>
     <row r="9">
@@ -1322,7 +1322,7 @@
         <v>57.58</v>
       </c>
       <c r="L9" t="n">
-        <v>51.82000000000001</v>
+        <v>51.82</v>
       </c>
     </row>
     <row r="10">
@@ -1362,7 +1362,7 @@
         <v>60.61</v>
       </c>
       <c r="L10" t="n">
-        <v>44.847</v>
+        <v>44.85</v>
       </c>
     </row>
     <row r="11">
@@ -1402,7 +1402,7 @@
         <v>51.85</v>
       </c>
       <c r="L11" t="n">
-        <v>46.668</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="12">
@@ -1412,37 +1412,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47.867</v>
+        <v>47.87</v>
       </c>
       <c r="C12" t="n">
-        <v>38.552</v>
+        <v>38.55</v>
       </c>
       <c r="D12" t="n">
-        <v>39.352</v>
+        <v>39.35</v>
       </c>
       <c r="E12" t="n">
-        <v>38.889</v>
+        <v>38.89</v>
       </c>
       <c r="F12" t="n">
-        <v>45.148</v>
+        <v>45.15</v>
       </c>
       <c r="G12" t="n">
-        <v>50.87499999999999</v>
+        <v>50.87</v>
       </c>
       <c r="H12" t="n">
-        <v>49.124</v>
+        <v>49.12</v>
       </c>
       <c r="I12" t="n">
-        <v>49.724</v>
+        <v>49.72</v>
       </c>
       <c r="J12" t="n">
-        <v>48.798</v>
+        <v>48.8</v>
       </c>
       <c r="K12" t="n">
-        <v>51.337</v>
+        <v>51.34</v>
       </c>
       <c r="L12" t="n">
-        <v>45.9666</v>
+        <v>45.97</v>
       </c>
     </row>
   </sheetData>
@@ -1593,7 +1593,7 @@
         <v>56.67</v>
       </c>
       <c r="L3" t="n">
-        <v>54.99899999999999</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -1633,7 +1633,7 @@
         <v>50</v>
       </c>
       <c r="L4" t="n">
-        <v>48.333</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="5">
@@ -1673,7 +1673,7 @@
         <v>50</v>
       </c>
       <c r="L5" t="n">
-        <v>50.33300000000001</v>
+        <v>50.33</v>
       </c>
     </row>
     <row r="6">
@@ -1713,7 +1713,7 @@
         <v>46.67</v>
       </c>
       <c r="L6" t="n">
-        <v>39.667</v>
+        <v>39.67</v>
       </c>
     </row>
     <row r="7">
@@ -1753,7 +1753,7 @@
         <v>66.67</v>
       </c>
       <c r="L7" t="n">
-        <v>51.66699999999999</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="8">
@@ -1793,7 +1793,7 @@
         <v>30</v>
       </c>
       <c r="L8" t="n">
-        <v>32.334</v>
+        <v>32.33</v>
       </c>
     </row>
     <row r="9">
@@ -1833,7 +1833,7 @@
         <v>56.67</v>
       </c>
       <c r="L9" t="n">
-        <v>46.666</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="10">
@@ -1873,7 +1873,7 @@
         <v>63.64</v>
       </c>
       <c r="L10" t="n">
-        <v>56.364</v>
+        <v>56.36</v>
       </c>
     </row>
     <row r="11">
@@ -1913,7 +1913,7 @@
         <v>57.58</v>
       </c>
       <c r="L11" t="n">
-        <v>49.395</v>
+        <v>49.4</v>
       </c>
     </row>
     <row r="12">
@@ -1923,37 +1923,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>49.059</v>
+        <v>49.06</v>
       </c>
       <c r="C12" t="n">
-        <v>43.849</v>
+        <v>43.85</v>
       </c>
       <c r="D12" t="n">
-        <v>42.81700000000001</v>
+        <v>42.82</v>
       </c>
       <c r="E12" t="n">
-        <v>38.544</v>
+        <v>38.54</v>
       </c>
       <c r="F12" t="n">
-        <v>44.847</v>
+        <v>44.85</v>
       </c>
       <c r="G12" t="n">
-        <v>51.36500000000001</v>
+        <v>51.37</v>
       </c>
       <c r="H12" t="n">
-        <v>50.243</v>
+        <v>50.24</v>
       </c>
       <c r="I12" t="n">
-        <v>53.758</v>
+        <v>53.76</v>
       </c>
       <c r="J12" t="n">
-        <v>53.819</v>
+        <v>53.82</v>
       </c>
       <c r="K12" t="n">
-        <v>53.45700000000001</v>
+        <v>53.46</v>
       </c>
       <c r="L12" t="n">
-        <v>48.1758</v>
+        <v>48.18</v>
       </c>
     </row>
   </sheetData>
@@ -2064,7 +2064,7 @@
         <v>60</v>
       </c>
       <c r="L2" t="n">
-        <v>47.667</v>
+        <v>47.67</v>
       </c>
     </row>
     <row r="3">
@@ -2104,7 +2104,7 @@
         <v>60</v>
       </c>
       <c r="L3" t="n">
-        <v>49.667</v>
+        <v>49.67</v>
       </c>
     </row>
     <row r="4">
@@ -2144,7 +2144,7 @@
         <v>43.33</v>
       </c>
       <c r="L4" t="n">
-        <v>35.666</v>
+        <v>35.67</v>
       </c>
     </row>
     <row r="5">
@@ -2184,7 +2184,7 @@
         <v>56.67</v>
       </c>
       <c r="L5" t="n">
-        <v>59.001</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -2224,7 +2224,7 @@
         <v>30</v>
       </c>
       <c r="L6" t="n">
-        <v>35.66699999999999</v>
+        <v>35.67</v>
       </c>
     </row>
     <row r="7">
@@ -2264,7 +2264,7 @@
         <v>60</v>
       </c>
       <c r="L7" t="n">
-        <v>52.001</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
@@ -2304,7 +2304,7 @@
         <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>41.66800000000001</v>
+        <v>41.67</v>
       </c>
     </row>
     <row r="9">
@@ -2344,7 +2344,7 @@
         <v>53.33</v>
       </c>
       <c r="L9" t="n">
-        <v>45.999</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10">
@@ -2384,7 +2384,7 @@
         <v>75.76000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>60.30499999999999</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="11">
@@ -2424,7 +2424,7 @@
         <v>48.48</v>
       </c>
       <c r="L11" t="n">
-        <v>46.966</v>
+        <v>46.97</v>
       </c>
     </row>
     <row r="12">
@@ -2437,34 +2437,34 @@
         <v>49.06</v>
       </c>
       <c r="C12" t="n">
-        <v>47.425</v>
+        <v>47.42</v>
       </c>
       <c r="D12" t="n">
-        <v>41.66699999999999</v>
+        <v>41.67</v>
       </c>
       <c r="E12" t="n">
-        <v>40.425</v>
+        <v>40.42</v>
       </c>
       <c r="F12" t="n">
-        <v>45.728</v>
+        <v>45.73</v>
       </c>
       <c r="G12" t="n">
-        <v>46.971</v>
+        <v>46.97</v>
       </c>
       <c r="H12" t="n">
-        <v>47.273</v>
+        <v>47.27</v>
       </c>
       <c r="I12" t="n">
-        <v>51.514</v>
+        <v>51.51</v>
       </c>
       <c r="J12" t="n">
-        <v>51.787</v>
+        <v>51.79</v>
       </c>
       <c r="K12" t="n">
-        <v>52.75699999999999</v>
+        <v>52.76</v>
       </c>
       <c r="L12" t="n">
-        <v>47.4607</v>
+        <v>47.46</v>
       </c>
     </row>
   </sheetData>
@@ -2478,7 +2478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2534,6 +2534,31 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>11_gaussians</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>12_gaussians</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>13_gaussians</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>14_gaussians</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>15_gaussians</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>mean</t>
         </is>
       </c>
@@ -2575,7 +2600,22 @@
         <v>63.33</v>
       </c>
       <c r="L2" t="n">
-        <v>56.33300000000001</v>
+        <v>63.33</v>
+      </c>
+      <c r="M2" t="n">
+        <v>60</v>
+      </c>
+      <c r="N2" t="n">
+        <v>63.33</v>
+      </c>
+      <c r="O2" t="n">
+        <v>63.33</v>
+      </c>
+      <c r="P2" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>58.22</v>
       </c>
     </row>
     <row r="3">
@@ -2615,7 +2655,22 @@
         <v>53.33</v>
       </c>
       <c r="L3" t="n">
-        <v>47.333</v>
+        <v>50</v>
+      </c>
+      <c r="M3" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="N3" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="O3" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="P3" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>47.56</v>
       </c>
     </row>
     <row r="4">
@@ -2655,7 +2710,22 @@
         <v>70</v>
       </c>
       <c r="L4" t="n">
-        <v>58</v>
+        <v>70</v>
+      </c>
+      <c r="M4" t="n">
+        <v>76.67</v>
+      </c>
+      <c r="N4" t="n">
+        <v>70</v>
+      </c>
+      <c r="O4" t="n">
+        <v>70</v>
+      </c>
+      <c r="P4" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>62.22</v>
       </c>
     </row>
     <row r="5">
@@ -2695,7 +2765,22 @@
         <v>46.67</v>
       </c>
       <c r="L5" t="n">
-        <v>47.999</v>
+        <v>46.67</v>
+      </c>
+      <c r="M5" t="n">
+        <v>50</v>
+      </c>
+      <c r="N5" t="n">
+        <v>53.33</v>
+      </c>
+      <c r="O5" t="n">
+        <v>50</v>
+      </c>
+      <c r="P5" t="n">
+        <v>46.67</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>48.44</v>
       </c>
     </row>
     <row r="6">
@@ -2735,7 +2820,22 @@
         <v>33.33</v>
       </c>
       <c r="L6" t="n">
-        <v>35.001</v>
+        <v>33.33</v>
+      </c>
+      <c r="M6" t="n">
+        <v>30</v>
+      </c>
+      <c r="N6" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="O6" t="n">
+        <v>33.33</v>
+      </c>
+      <c r="P6" t="n">
+        <v>36.67</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>34.44</v>
       </c>
     </row>
     <row r="7">
@@ -2775,7 +2875,22 @@
         <v>63.33</v>
       </c>
       <c r="L7" t="n">
-        <v>49.667</v>
+        <v>60</v>
+      </c>
+      <c r="M7" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="N7" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="O7" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="P7" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>54.89</v>
       </c>
     </row>
     <row r="8">
@@ -2815,7 +2930,22 @@
         <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>44.001</v>
+        <v>40</v>
+      </c>
+      <c r="M8" t="n">
+        <v>40</v>
+      </c>
+      <c r="N8" t="n">
+        <v>40</v>
+      </c>
+      <c r="O8" t="n">
+        <v>40</v>
+      </c>
+      <c r="P8" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>42.67</v>
       </c>
     </row>
     <row r="9">
@@ -2855,7 +2985,22 @@
         <v>66.67</v>
       </c>
       <c r="L9" t="n">
-        <v>59.09399999999999</v>
+        <v>60.61</v>
+      </c>
+      <c r="M9" t="n">
+        <v>57.58</v>
+      </c>
+      <c r="N9" t="n">
+        <v>63.64</v>
+      </c>
+      <c r="O9" t="n">
+        <v>60.61</v>
+      </c>
+      <c r="P9" t="n">
+        <v>57.58</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>59.4</v>
       </c>
     </row>
     <row r="10">
@@ -2895,7 +3040,22 @@
         <v>66.67</v>
       </c>
       <c r="L10" t="n">
-        <v>58.974</v>
+        <v>66.67</v>
+      </c>
+      <c r="M10" t="n">
+        <v>56.41</v>
+      </c>
+      <c r="N10" t="n">
+        <v>58.97</v>
+      </c>
+      <c r="O10" t="n">
+        <v>66.67</v>
+      </c>
+      <c r="P10" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>60.17</v>
       </c>
     </row>
     <row r="11">
@@ -2935,7 +3095,22 @@
         <v>59.26</v>
       </c>
       <c r="L11" t="n">
-        <v>49.63</v>
+        <v>51.85</v>
+      </c>
+      <c r="M11" t="n">
+        <v>51.85</v>
+      </c>
+      <c r="N11" t="n">
+        <v>55.56</v>
+      </c>
+      <c r="O11" t="n">
+        <v>48.15</v>
+      </c>
+      <c r="P11" t="n">
+        <v>59.26</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>50.86</v>
       </c>
     </row>
     <row r="12">
@@ -2945,37 +3120,52 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>49.45700000000001</v>
+        <v>49.46</v>
       </c>
       <c r="C12" t="n">
-        <v>43.09699999999999</v>
+        <v>43.1</v>
       </c>
       <c r="D12" t="n">
-        <v>49.42899999999999</v>
+        <v>49.43</v>
       </c>
       <c r="E12" t="n">
-        <v>42.35299999999999</v>
+        <v>42.35</v>
       </c>
       <c r="F12" t="n">
-        <v>50.883</v>
+        <v>50.88</v>
       </c>
       <c r="G12" t="n">
-        <v>53.355</v>
+        <v>53.36</v>
       </c>
       <c r="H12" t="n">
-        <v>52.496</v>
+        <v>52.5</v>
       </c>
       <c r="I12" t="n">
-        <v>54.26000000000001</v>
+        <v>54.26</v>
       </c>
       <c r="J12" t="n">
-        <v>54.443</v>
+        <v>54.44</v>
       </c>
       <c r="K12" t="n">
-        <v>56.259</v>
+        <v>56.26</v>
       </c>
       <c r="L12" t="n">
-        <v>50.6032</v>
+        <v>54.25</v>
+      </c>
+      <c r="M12" t="n">
+        <v>53.58</v>
+      </c>
+      <c r="N12" t="n">
+        <v>55.15</v>
+      </c>
+      <c r="O12" t="n">
+        <v>54.54</v>
+      </c>
+      <c r="P12" t="n">
+        <v>54.76</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>51.89</v>
       </c>
     </row>
   </sheetData>
@@ -3086,7 +3276,7 @@
         <v>56.67</v>
       </c>
       <c r="L2" t="n">
-        <v>51.335</v>
+        <v>51.34</v>
       </c>
     </row>
     <row r="3">
@@ -3126,7 +3316,7 @@
         <v>50</v>
       </c>
       <c r="L3" t="n">
-        <v>51.33299999999999</v>
+        <v>51.33</v>
       </c>
     </row>
     <row r="4">
@@ -3166,7 +3356,7 @@
         <v>56.67</v>
       </c>
       <c r="L4" t="n">
-        <v>50.667</v>
+        <v>50.67</v>
       </c>
     </row>
     <row r="5">
@@ -3206,7 +3396,7 @@
         <v>50</v>
       </c>
       <c r="L5" t="n">
-        <v>49.999</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -3246,7 +3436,7 @@
         <v>36.67</v>
       </c>
       <c r="L6" t="n">
-        <v>43.334</v>
+        <v>43.33</v>
       </c>
     </row>
     <row r="7">
@@ -3286,7 +3476,7 @@
         <v>60</v>
       </c>
       <c r="L7" t="n">
-        <v>45.999</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -3326,7 +3516,7 @@
         <v>36.67</v>
       </c>
       <c r="L8" t="n">
-        <v>37.333</v>
+        <v>37.33</v>
       </c>
     </row>
     <row r="9">
@@ -3366,7 +3556,7 @@
         <v>51.52</v>
       </c>
       <c r="L9" t="n">
-        <v>47.273</v>
+        <v>47.27</v>
       </c>
     </row>
     <row r="10">
@@ -3406,7 +3596,7 @@
         <v>58.97</v>
       </c>
       <c r="L10" t="n">
-        <v>54.358</v>
+        <v>54.36</v>
       </c>
     </row>
     <row r="11">
@@ -3446,7 +3636,7 @@
         <v>44.44</v>
       </c>
       <c r="L11" t="n">
-        <v>48.517</v>
+        <v>48.52</v>
       </c>
     </row>
     <row r="12">
@@ -3456,37 +3646,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47.896</v>
+        <v>47.9</v>
       </c>
       <c r="C12" t="n">
         <v>44.5</v>
       </c>
       <c r="D12" t="n">
-        <v>44.134</v>
+        <v>44.13</v>
       </c>
       <c r="E12" t="n">
-        <v>39.356</v>
+        <v>39.36</v>
       </c>
       <c r="F12" t="n">
-        <v>52.033</v>
+        <v>52.03</v>
       </c>
       <c r="G12" t="n">
-        <v>51.81700000000001</v>
+        <v>51.82</v>
       </c>
       <c r="H12" t="n">
-        <v>50.75099999999999</v>
+        <v>50.75</v>
       </c>
       <c r="I12" t="n">
-        <v>48.923</v>
+        <v>48.92</v>
       </c>
       <c r="J12" t="n">
-        <v>50.577</v>
+        <v>50.58</v>
       </c>
       <c r="K12" t="n">
-        <v>50.16100000000001</v>
+        <v>50.16</v>
       </c>
       <c r="L12" t="n">
-        <v>48.0148</v>
+        <v>48.01</v>
       </c>
     </row>
   </sheetData>
@@ -3597,7 +3787,7 @@
         <v>56.67</v>
       </c>
       <c r="L2" t="n">
-        <v>51.334</v>
+        <v>51.33</v>
       </c>
     </row>
     <row r="3">
@@ -3637,7 +3827,7 @@
         <v>46.67</v>
       </c>
       <c r="L3" t="n">
-        <v>45.333</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="4">
@@ -3717,7 +3907,7 @@
         <v>43.33</v>
       </c>
       <c r="L5" t="n">
-        <v>44.667</v>
+        <v>44.67</v>
       </c>
     </row>
     <row r="6">
@@ -3757,7 +3947,7 @@
         <v>56.67</v>
       </c>
       <c r="L6" t="n">
-        <v>46.666</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="7">
@@ -3797,7 +3987,7 @@
         <v>56.67</v>
       </c>
       <c r="L7" t="n">
-        <v>50.335</v>
+        <v>50.34</v>
       </c>
     </row>
     <row r="8">
@@ -3837,7 +4027,7 @@
         <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>41.66499999999999</v>
+        <v>41.66</v>
       </c>
     </row>
     <row r="9">
@@ -3877,7 +4067,7 @@
         <v>54.55</v>
       </c>
       <c r="L9" t="n">
-        <v>49.393</v>
+        <v>49.39</v>
       </c>
     </row>
     <row r="10">
@@ -3917,7 +4107,7 @@
         <v>51.28</v>
       </c>
       <c r="L10" t="n">
-        <v>51.794</v>
+        <v>51.79</v>
       </c>
     </row>
     <row r="11">
@@ -3957,7 +4147,7 @@
         <v>44.44</v>
       </c>
       <c r="L11" t="n">
-        <v>48.889</v>
+        <v>48.89</v>
       </c>
     </row>
     <row r="12">
@@ -3967,37 +4157,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47.152</v>
+        <v>47.15</v>
       </c>
       <c r="C12" t="n">
-        <v>44.79799999999999</v>
+        <v>44.8</v>
       </c>
       <c r="D12" t="n">
         <v>43.42</v>
       </c>
       <c r="E12" t="n">
-        <v>41.598</v>
+        <v>41.6</v>
       </c>
       <c r="F12" t="n">
-        <v>52.621</v>
+        <v>52.62</v>
       </c>
       <c r="G12" t="n">
-        <v>50.16699999999999</v>
+        <v>50.17</v>
       </c>
       <c r="H12" t="n">
-        <v>46.652</v>
+        <v>46.65</v>
       </c>
       <c r="I12" t="n">
-        <v>50.164</v>
+        <v>50.16</v>
       </c>
       <c r="J12" t="n">
-        <v>50.476</v>
+        <v>50.48</v>
       </c>
       <c r="K12" t="n">
-        <v>51.02800000000001</v>
+        <v>51.03</v>
       </c>
       <c r="L12" t="n">
-        <v>47.8076</v>
+        <v>47.81</v>
       </c>
     </row>
   </sheetData>
@@ -4108,7 +4298,7 @@
         <v>53.33</v>
       </c>
       <c r="L2" t="n">
-        <v>48.666</v>
+        <v>48.67</v>
       </c>
     </row>
     <row r="3">
@@ -4148,7 +4338,7 @@
         <v>53.33</v>
       </c>
       <c r="L3" t="n">
-        <v>51.66700000000001</v>
+        <v>51.67</v>
       </c>
     </row>
     <row r="4">
@@ -4188,7 +4378,7 @@
         <v>56.67</v>
       </c>
       <c r="L4" t="n">
-        <v>54.99799999999999</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -4228,7 +4418,7 @@
         <v>46.67</v>
       </c>
       <c r="L5" t="n">
-        <v>44.999</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -4268,7 +4458,7 @@
         <v>60</v>
       </c>
       <c r="L6" t="n">
-        <v>48.333</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="7">
@@ -4308,7 +4498,7 @@
         <v>56.67</v>
       </c>
       <c r="L7" t="n">
-        <v>48.334</v>
+        <v>48.33</v>
       </c>
     </row>
     <row r="8">
@@ -4348,7 +4538,7 @@
         <v>40</v>
       </c>
       <c r="L8" t="n">
-        <v>45.333</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="9">
@@ -4388,7 +4578,7 @@
         <v>60.61</v>
       </c>
       <c r="L9" t="n">
-        <v>59.09400000000001</v>
+        <v>59.09</v>
       </c>
     </row>
     <row r="10">
@@ -4428,7 +4618,7 @@
         <v>53.85</v>
       </c>
       <c r="L10" t="n">
-        <v>55.898</v>
+        <v>55.9</v>
       </c>
     </row>
     <row r="11">
@@ -4468,7 +4658,7 @@
         <v>37.04</v>
       </c>
       <c r="L11" t="n">
-        <v>35.185</v>
+        <v>35.18</v>
       </c>
     </row>
     <row r="12">
@@ -4478,37 +4668,37 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>46.54499999999999</v>
+        <v>46.54</v>
       </c>
       <c r="C12" t="n">
-        <v>41.669</v>
+        <v>41.67</v>
       </c>
       <c r="D12" t="n">
-        <v>44.588</v>
+        <v>44.59</v>
       </c>
       <c r="E12" t="n">
-        <v>44.796</v>
+        <v>44.8</v>
       </c>
       <c r="F12" t="n">
-        <v>55.527</v>
+        <v>55.53</v>
       </c>
       <c r="G12" t="n">
-        <v>53.96700000000001</v>
+        <v>53.97</v>
       </c>
       <c r="H12" t="n">
-        <v>51.65500000000001</v>
+        <v>51.66</v>
       </c>
       <c r="I12" t="n">
-        <v>49.47600000000001</v>
+        <v>49.48</v>
       </c>
       <c r="J12" t="n">
-        <v>52.467</v>
+        <v>52.47</v>
       </c>
       <c r="K12" t="n">
-        <v>51.81699999999999</v>
+        <v>51.82</v>
       </c>
       <c r="L12" t="n">
-        <v>49.2507</v>
+        <v>49.25</v>
       </c>
     </row>
   </sheetData>
@@ -4619,7 +4809,7 @@
         <v>56.67</v>
       </c>
       <c r="L2" t="n">
-        <v>45.33300000000001</v>
+        <v>45.33</v>
       </c>
     </row>
     <row r="3">
@@ -4659,7 +4849,7 @@
         <v>53.33</v>
       </c>
       <c r="L3" t="n">
-        <v>48.999</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -4699,7 +4889,7 @@
         <v>53.33</v>
       </c>
       <c r="L4" t="n">
-        <v>49.667</v>
+        <v>49.67</v>
       </c>
     </row>
     <row r="5">
@@ -4739,7 +4929,7 @@
         <v>50</v>
       </c>
       <c r="L5" t="n">
-        <v>44.333</v>
+        <v>44.33</v>
       </c>
     </row>
     <row r="6">
@@ -4779,7 +4969,7 @@
         <v>66.67</v>
       </c>
       <c r="L6" t="n">
-        <v>48.666</v>
+        <v>48.67</v>
       </c>
     </row>
     <row r="7">
@@ -4819,7 +5009,7 @@
         <v>56.67</v>
       </c>
       <c r="L7" t="n">
-        <v>47.334</v>
+        <v>47.33</v>
       </c>
     </row>
     <row r="8">
@@ -4859,7 +5049,7 @@
         <v>46.67</v>
       </c>
       <c r="L8" t="n">
-        <v>41.001</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
@@ -4899,7 +5089,7 @@
         <v>57.58</v>
       </c>
       <c r="L9" t="n">
-        <v>55.15400000000001</v>
+        <v>55.15</v>
       </c>
     </row>
     <row r="10">
@@ -4939,7 +5129,7 @@
         <v>64.09999999999999</v>
       </c>
       <c r="L10" t="n">
-        <v>46.666</v>
+        <v>46.67</v>
       </c>
     </row>
     <row r="11">
@@ -4979,7 +5169,7 @@
         <v>37.04</v>
       </c>
       <c r="L11" t="n">
-        <v>42.593</v>
+        <v>42.59</v>
       </c>
     </row>
     <row r="12">
@@ -4989,25 +5179,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>46.002</v>
+        <v>46</v>
       </c>
       <c r="C12" t="n">
-        <v>41.47799999999999</v>
+        <v>41.48</v>
       </c>
       <c r="D12" t="n">
-        <v>42.719</v>
+        <v>42.72</v>
       </c>
       <c r="E12" t="n">
-        <v>40.658</v>
+        <v>40.66</v>
       </c>
       <c r="F12" t="n">
-        <v>48.42299999999999</v>
+        <v>48.42</v>
       </c>
       <c r="G12" t="n">
         <v>48.3</v>
       </c>
       <c r="H12" t="n">
-        <v>49.26000000000001</v>
+        <v>49.26</v>
       </c>
       <c r="I12" t="n">
         <v>47.96</v>
@@ -5016,10 +5206,10 @@
         <v>50.74</v>
       </c>
       <c r="K12" t="n">
-        <v>54.206</v>
+        <v>54.21</v>
       </c>
       <c r="L12" t="n">
-        <v>46.9746</v>
+        <v>46.97</v>
       </c>
     </row>
   </sheetData>
@@ -5130,7 +5320,7 @@
         <v>63.33</v>
       </c>
       <c r="L2" t="n">
-        <v>56.33300000000001</v>
+        <v>56.33</v>
       </c>
     </row>
     <row r="3">
@@ -5170,7 +5360,7 @@
         <v>43.33</v>
       </c>
       <c r="L3" t="n">
-        <v>50.332</v>
+        <v>50.33</v>
       </c>
     </row>
     <row r="4">
@@ -5210,7 +5400,7 @@
         <v>36.67</v>
       </c>
       <c r="L4" t="n">
-        <v>35.001</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -5250,7 +5440,7 @@
         <v>63.33</v>
       </c>
       <c r="L5" t="n">
-        <v>51.33300000000001</v>
+        <v>51.33</v>
       </c>
     </row>
     <row r="6">
@@ -5290,7 +5480,7 @@
         <v>50</v>
       </c>
       <c r="L6" t="n">
-        <v>41.335</v>
+        <v>41.34</v>
       </c>
     </row>
     <row r="7">
@@ -5330,7 +5520,7 @@
         <v>60</v>
       </c>
       <c r="L7" t="n">
-        <v>53.66800000000001</v>
+        <v>53.67</v>
       </c>
     </row>
     <row r="8">
@@ -5370,7 +5560,7 @@
         <v>36.67</v>
       </c>
       <c r="L8" t="n">
-        <v>45.667</v>
+        <v>45.67</v>
       </c>
     </row>
     <row r="9">
@@ -5410,7 +5600,7 @@
         <v>63.64</v>
       </c>
       <c r="L9" t="n">
-        <v>53.032</v>
+        <v>53.03</v>
       </c>
     </row>
     <row r="10">
@@ -5450,7 +5640,7 @@
         <v>51.52</v>
       </c>
       <c r="L10" t="n">
-        <v>43.33399999999999</v>
+        <v>43.33</v>
       </c>
     </row>
     <row r="11">
@@ -5503,34 +5693,34 @@
         <v>49.2</v>
       </c>
       <c r="C12" t="n">
-        <v>41.929</v>
+        <v>41.93</v>
       </c>
       <c r="D12" t="n">
         <v>42.28</v>
       </c>
       <c r="E12" t="n">
-        <v>38.719</v>
+        <v>38.72</v>
       </c>
       <c r="F12" t="n">
-        <v>46.573</v>
+        <v>46.57</v>
       </c>
       <c r="G12" t="n">
-        <v>51.361</v>
+        <v>51.36</v>
       </c>
       <c r="H12" t="n">
-        <v>49.414</v>
+        <v>49.41</v>
       </c>
       <c r="I12" t="n">
-        <v>50.022</v>
+        <v>50.02</v>
       </c>
       <c r="J12" t="n">
-        <v>50.354</v>
+        <v>50.35</v>
       </c>
       <c r="K12" t="n">
-        <v>51.29300000000001</v>
+        <v>51.29</v>
       </c>
       <c r="L12" t="n">
-        <v>47.11450000000001</v>
+        <v>47.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>